<commit_message>
update CVs and common ontologies to new model
</commit_message>
<xml_diff>
--- a/SR-dev/metadata/cv-skos-play.xlsx
+++ b/SR-dev/metadata/cv-skos-play.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwceur.sharepoint.com/teams/BE-T88621b17cfcd4658ab5f9764b8a23150/Shared Documents/General/Task 07 - Creation, maintenance and packaging of tools/A07.01 Semantic Registry/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aschiltz003\Documents\GitHub\EU-wide-Registry-of-Semantic-Models\SR-dev\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="256" documentId="13_ncr:1_{2753F300-8B54-4511-9600-487CDA069158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0727227E-1633-4998-88C1-20BB245C5653}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9EFBFF-7321-49EE-8948-B82E67A005F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-75" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Standard" sheetId="2" r:id="rId1"/>
+    <sheet name="Asset" sheetId="2" r:id="rId1"/>
     <sheet name="Agent" sheetId="4" r:id="rId2"/>
     <sheet name="Class" sheetId="5" r:id="rId3"/>
     <sheet name="ContactPoint" sheetId="6" r:id="rId4"/>
     <sheet name="Document" sheetId="7" r:id="rId5"/>
     <sheet name="Location" sheetId="8" r:id="rId6"/>
-    <sheet name="ResourceDescriptor" sheetId="9" r:id="rId7"/>
+    <sheet name="AssetDistribution" sheetId="9" r:id="rId7"/>
     <sheet name="Concept" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
@@ -48,7 +48,7 @@
     <author>tc={69670AD0-6484-4FFE-A455-3E1E94647EC3}</author>
   </authors>
   <commentList>
-    <comment ref="L14" authorId="0" shapeId="0" xr:uid="{69670AD0-6484-4FFE-A455-3E1E94647EC3}">
+    <comment ref="K15" authorId="0" shapeId="0" xr:uid="{69670AD0-6484-4FFE-A455-3E1E94647EC3}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -61,14 +61,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="195">
   <si>
     <t>ConceptScheme URI</t>
   </si>
   <si>
-    <t>http://purl.org/dc/terms/Standard</t>
-  </si>
-  <si>
     <t>PREFIX</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
     <t>cv:hasImplementation</t>
   </si>
   <si>
-    <t>dct:hasPart</t>
-  </si>
-  <si>
     <t>foaf:homepage</t>
   </si>
   <si>
@@ -264,9 +258,6 @@
     <t>dct:Location</t>
   </si>
   <si>
-    <t>http://www.w3.org/ns/dx/prof/ResourceDescriptor</t>
-  </si>
-  <si>
     <t>skos</t>
   </si>
   <si>
@@ -303,9 +294,6 @@
     <t>dct:description@en</t>
   </si>
   <si>
-    <t>locn:Address,cv:ContactPoint,adms:Identifier,dct:Location,person:Person</t>
-  </si>
-  <si>
     <t>locn:Address</t>
   </si>
   <si>
@@ -381,9 +369,6 @@
     <t>CLV</t>
   </si>
   <si>
-    <t>locn:Address,cv:AdminUnit,locn:Geometry,dct:Location,ad:LocatorDesignator</t>
-  </si>
-  <si>
     <t>2.2.0</t>
   </si>
   <si>
@@ -417,9 +402,6 @@
     <t>Legal Entity</t>
   </si>
   <si>
-    <t>cv:AccountingDocument,locn:Address,cv:ContactPoint,adms:Identifier,legal:LegalEntity</t>
-  </si>
-  <si>
     <t>https://semiceu.github.io/Core-Business-Vocabulary/releases/2.2.0/voc/core-business-ap.ttl</t>
   </si>
   <si>
@@ -492,9 +474,6 @@
     <t>Requirement</t>
   </si>
   <si>
-    <t>cv:Constraint,cv:Criterion,cv:Evidence,cv:EvidenceType,cv:EvidenceTypeList,cv:InformationConcept,cv:InformationRequirement,cv:ReferenceFramework,cv:Requirement</t>
-  </si>
-  <si>
     <t>https://semiceu.github.io/CCCEV/releases/2.1.0/voc/cccev.ttl</t>
   </si>
   <si>
@@ -525,9 +504,6 @@
     <t>Public Organisation</t>
   </si>
   <si>
-    <t>locn:Address,cv:ContactPoint,adms:Identifier,cv:PublicOrganisation</t>
-  </si>
-  <si>
     <t>https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
   </si>
   <si>
@@ -561,9 +537,6 @@
     <t>Public Event</t>
   </si>
   <si>
-    <t>locn:Address,cv:ContactPoint,cv:Participation,cv:PublicEvent</t>
-  </si>
-  <si>
     <t>cb</t>
   </si>
   <si>
@@ -576,9 +549,6 @@
     <t>http://publications.europa.eu/resource/authority/country/EUR</t>
   </si>
   <si>
-    <t>prof:ResourceDescriptor</t>
-  </si>
-  <si>
     <t>http://publications.europa.eu/resource/authority/file-type/RDF_TURTLE</t>
   </si>
   <si>
@@ -651,7 +621,31 @@
     <t>https://semiceu.github.io/CPOV/releases/2.1.1/voc/core-public-organisation</t>
   </si>
   <si>
-    <t>prof:hasResource</t>
+    <t>http://www.w3.org/ns/adms#Asset</t>
+  </si>
+  <si>
+    <t>amds:AssetDistribution</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/adms#AssetDistribution</t>
+  </si>
+  <si>
+    <t>dcat:distribution</t>
+  </si>
+  <si>
+    <t>rdfs:isDefinedBy</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Location-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV, https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV, https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Location-Vocabulary/</t>
   </si>
 </sst>
 </file>
@@ -710,7 +704,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -728,7 +722,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1040,7 +1033,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="L14" dT="2025-05-08T09:36:43.81" personId="{FC617CA1-A774-4F32-AB9B-CEA632C8D8C7}" id="{69670AD0-6484-4FFE-A455-3E1E94647EC3}">
+  <threadedComment ref="K15" dT="2025-05-08T09:36:43.81" personId="{FC617CA1-A774-4F32-AB9B-CEA632C8D8C7}" id="{69670AD0-6484-4FFE-A455-3E1E94647EC3}">
     <text>To be added</text>
   </threadedComment>
 </ThreadedComments>
@@ -1048,7 +1041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Y20"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50.33203125" customWidth="1"/>
@@ -1060,498 +1053,505 @@
     <col min="7" max="7" width="11.6640625" customWidth="1"/>
     <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.109375" customWidth="1"/>
-    <col min="10" max="10" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.88671875" customWidth="1"/>
-    <col min="12" max="12" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.88671875" customWidth="1"/>
-    <col min="15" max="15" width="12.5546875" customWidth="1"/>
-    <col min="16" max="16" width="58.5546875" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" customWidth="1"/>
-    <col min="18" max="18" width="27.33203125" customWidth="1"/>
-    <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="11" customWidth="1"/>
-    <col min="21" max="21" width="11.109375" customWidth="1"/>
-    <col min="22" max="22" width="10.6640625" customWidth="1"/>
-    <col min="23" max="23" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
+    <col min="11" max="11" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.88671875" customWidth="1"/>
+    <col min="14" max="14" width="12.5546875" customWidth="1"/>
+    <col min="15" max="15" width="58.5546875" customWidth="1"/>
+    <col min="16" max="16" width="9.6640625" customWidth="1"/>
+    <col min="17" max="17" width="27.33203125" customWidth="1"/>
+    <col min="18" max="18" width="12" customWidth="1"/>
+    <col min="19" max="19" width="11" customWidth="1"/>
+    <col min="20" max="20" width="11.109375" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" customWidth="1"/>
+    <col min="22" max="22" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H15" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="J15" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="L15" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="L14" s="2" t="s">
+      <c r="N15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="M14" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="N14" s="2" t="s">
+      <c r="O15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="O14" s="2" t="s">
+      <c r="P15" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P14" s="2" t="s">
+      <c r="Q15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="R15" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="Q14" s="2" t="s">
+      <c r="S15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="R14" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="S14" s="2" t="s">
+      <c r="T15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="T14" s="2" t="s">
+      <c r="U15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="U14" s="2" t="s">
+      <c r="V15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="W15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="V14" s="2" t="s">
+      <c r="X15" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>39</v>
       </c>
-      <c r="W14" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="X14" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y14" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" t="s">
-        <v>169</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" t="s">
-        <v>169</v>
-      </c>
-      <c r="E15" s="5">
-        <f>DATE(2024,5,6)</f>
-        <v>45418</v>
-      </c>
-      <c r="H15" t="s">
-        <v>42</v>
-      </c>
-      <c r="J15" t="s">
-        <v>80</v>
-      </c>
-      <c r="K15" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="L15" t="s">
-        <v>64</v>
-      </c>
-      <c r="M15" t="s">
-        <v>89</v>
-      </c>
-      <c r="P15" t="s">
-        <v>183</v>
-      </c>
-      <c r="S15" t="s">
-        <v>169</v>
-      </c>
-      <c r="W15" t="s">
-        <v>43</v>
-      </c>
-      <c r="X15" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>90</v>
-      </c>
       <c r="B16" t="s">
-        <v>169</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="C16" s="1"/>
       <c r="D16" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="E16" s="5">
         <f>DATE(2024,5,6)</f>
         <v>45418</v>
       </c>
       <c r="H16" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="J16" t="s">
-        <v>106</v>
-      </c>
-      <c r="K16" s="9" t="s">
-        <v>191</v>
+        <v>180</v>
+      </c>
+      <c r="K16" t="s">
+        <v>62</v>
       </c>
       <c r="L16" t="s">
-        <v>178</v>
-      </c>
-      <c r="M16" t="s">
-        <v>105</v>
-      </c>
-      <c r="P16" t="s">
-        <v>183</v>
-      </c>
-      <c r="S16" t="s">
-        <v>169</v>
+        <v>85</v>
+      </c>
+      <c r="O16" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>3</v>
+      </c>
+      <c r="R16" t="s">
+        <v>160</v>
+      </c>
+      <c r="V16" t="s">
+        <v>41</v>
       </c>
       <c r="W16" t="s">
-        <v>103</v>
+        <v>42</v>
       </c>
       <c r="X16" t="s">
-        <v>104</v>
-      </c>
-      <c r="Y16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>86</v>
       </c>
       <c r="B17" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D17" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="E17" s="5">
         <f>DATE(2024,5,6)</f>
         <v>45418</v>
       </c>
       <c r="H17" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="J17" t="s">
-        <v>118</v>
-      </c>
-      <c r="K17" s="9" t="s">
-        <v>194</v>
+        <v>181</v>
+      </c>
+      <c r="K17" t="s">
+        <v>168</v>
       </c>
       <c r="L17" t="s">
-        <v>179</v>
-      </c>
-      <c r="M17" t="s">
-        <v>109</v>
-      </c>
-      <c r="P17" t="s">
-        <v>183</v>
-      </c>
-      <c r="S17" t="s">
-        <v>169</v>
+        <v>101</v>
+      </c>
+      <c r="O17" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>3</v>
+      </c>
+      <c r="R17" t="s">
+        <v>160</v>
+      </c>
+      <c r="V17" t="s">
+        <v>99</v>
       </c>
       <c r="W17" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="X17" t="s">
-        <v>107</v>
-      </c>
-      <c r="Y17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="B18" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D18" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="E18" s="5">
         <f>DATE(2024,5,6)</f>
         <v>45418</v>
       </c>
       <c r="H18" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="J18" t="s">
-        <v>143</v>
-      </c>
-      <c r="K18" s="9" t="s">
-        <v>192</v>
+        <v>184</v>
+      </c>
+      <c r="K18" t="s">
+        <v>169</v>
       </c>
       <c r="L18" t="s">
-        <v>180</v>
-      </c>
-      <c r="M18" t="s">
-        <v>122</v>
-      </c>
-      <c r="P18" t="s">
-        <v>183</v>
-      </c>
-      <c r="S18" t="s">
-        <v>169</v>
+        <v>104</v>
+      </c>
+      <c r="O18" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>3</v>
+      </c>
+      <c r="R18" t="s">
+        <v>160</v>
+      </c>
+      <c r="V18" t="s">
+        <v>103</v>
       </c>
       <c r="W18" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="X18" t="s">
-        <v>104</v>
-      </c>
-      <c r="Y18" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="B19" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D19" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="E19" s="5">
         <f>DATE(2024,5,6)</f>
         <v>45418</v>
       </c>
       <c r="H19" t="s">
+        <v>118</v>
+      </c>
+      <c r="J19" t="s">
+        <v>182</v>
+      </c>
+      <c r="K19" t="s">
+        <v>170</v>
+      </c>
+      <c r="L19" t="s">
+        <v>116</v>
+      </c>
+      <c r="O19" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>3</v>
+      </c>
+      <c r="R19" t="s">
+        <v>160</v>
+      </c>
+      <c r="V19" t="s">
+        <v>117</v>
+      </c>
+      <c r="W19" t="s">
+        <v>100</v>
+      </c>
+      <c r="X19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>139</v>
+      </c>
+      <c r="B20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D20" t="s">
+        <v>160</v>
+      </c>
+      <c r="E20" s="5">
+        <f>DATE(2024,5,6)</f>
+        <v>45418</v>
+      </c>
+      <c r="H20" t="s">
+        <v>140</v>
+      </c>
+      <c r="J20" t="s">
+        <v>185</v>
+      </c>
+      <c r="K20" t="s">
+        <v>171</v>
+      </c>
+      <c r="L20" t="s">
+        <v>141</v>
+      </c>
+      <c r="O20" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>3</v>
+      </c>
+      <c r="R20" t="s">
+        <v>160</v>
+      </c>
+      <c r="V20" t="s">
+        <v>142</v>
+      </c>
+      <c r="W20" t="s">
+        <v>42</v>
+      </c>
+      <c r="X20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>147</v>
       </c>
-      <c r="J19" t="s">
-        <v>154</v>
-      </c>
-      <c r="K19" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="L19" t="s">
-        <v>181</v>
-      </c>
-      <c r="M19" t="s">
+      <c r="B21" t="s">
+        <v>160</v>
+      </c>
+      <c r="D21" t="s">
+        <v>160</v>
+      </c>
+      <c r="E21" s="5">
+        <f t="shared" ref="E21" si="0">DATE(2024,5,6)</f>
+        <v>45418</v>
+      </c>
+      <c r="H21" t="s">
         <v>148</v>
       </c>
-      <c r="P19" t="s">
+      <c r="J21" t="s">
         <v>183</v>
       </c>
-      <c r="S19" t="s">
-        <v>169</v>
-      </c>
-      <c r="W19" t="s">
-        <v>149</v>
-      </c>
-      <c r="X19" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20" t="s">
-        <v>169</v>
-      </c>
-      <c r="D20" t="s">
-        <v>169</v>
-      </c>
-      <c r="E20" s="5">
-        <f t="shared" ref="E20" si="0">DATE(2024,5,6)</f>
-        <v>45418</v>
-      </c>
-      <c r="H20" t="s">
-        <v>156</v>
-      </c>
-      <c r="J20" t="s">
-        <v>166</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="L20" t="s">
-        <v>182</v>
-      </c>
-      <c r="M20" t="s">
-        <v>158</v>
-      </c>
-      <c r="P20" t="s">
-        <v>183</v>
-      </c>
-      <c r="S20" t="s">
-        <v>169</v>
-      </c>
-      <c r="W20" t="s">
-        <v>159</v>
-      </c>
-      <c r="X20" t="s">
+      <c r="K21" t="s">
+        <v>172</v>
+      </c>
+      <c r="L21" t="s">
+        <v>150</v>
+      </c>
+      <c r="O21" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>3</v>
+      </c>
+      <c r="R21" t="s">
         <v>160</v>
       </c>
-      <c r="Y20" t="s">
-        <v>74</v>
+      <c r="V21" t="s">
+        <v>151</v>
+      </c>
+      <c r="W21" t="s">
+        <v>152</v>
+      </c>
+      <c r="X21" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1575,142 +1575,142 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
         <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
         <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
       </c>
       <c r="D12" s="1"/>
     </row>
@@ -1719,33 +1719,33 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1761,461 +1761,531 @@
     <col min="1" max="1" width="31.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.109375" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="7" max="8" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C4" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
         <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
         <v>5</v>
-      </c>
-      <c r="C7" t="s">
-        <v>6</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
         <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
         <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>16</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
         <v>19</v>
-      </c>
-      <c r="C13" t="s">
-        <v>20</v>
       </c>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" t="s">
         <v>11</v>
-      </c>
-      <c r="C16" t="s">
-        <v>12</v>
       </c>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
         <v>17</v>
-      </c>
-      <c r="C17" t="s">
-        <v>18</v>
       </c>
       <c r="D17" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D20" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D21" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C22" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D22" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D23" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B25" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D25" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B26" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D26" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B27" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D27" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C28" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D28" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B29" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C29" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D29" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C30" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D30" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B31" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C31" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D31" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>123</v>
+      </c>
+      <c r="B32" t="s">
+        <v>124</v>
+      </c>
+      <c r="C32" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>125</v>
+      </c>
+      <c r="B33" t="s">
+        <v>126</v>
+      </c>
+      <c r="C33" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>127</v>
+      </c>
+      <c r="B34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>129</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B35" t="s">
         <v>130</v>
       </c>
-      <c r="C32" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="C35" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>131</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B36" t="s">
         <v>132</v>
       </c>
-      <c r="C33" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+      <c r="C36" t="s">
+        <v>80</v>
+      </c>
+      <c r="D36" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>133</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B37" t="s">
         <v>134</v>
       </c>
-      <c r="C34" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="C37" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
         <v>135</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B38" t="s">
         <v>136</v>
       </c>
-      <c r="C35" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>137</v>
-      </c>
-      <c r="B36" t="s">
-        <v>138</v>
-      </c>
-      <c r="C36" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="C38" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" t="s">
+        <v>146</v>
+      </c>
+      <c r="C39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D39" t="s">
         <v>139</v>
       </c>
-      <c r="B37" t="s">
-        <v>140</v>
-      </c>
-      <c r="C37" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>141</v>
-      </c>
-      <c r="B38" t="s">
-        <v>142</v>
-      </c>
-      <c r="C38" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>152</v>
-      </c>
-      <c r="B39" t="s">
-        <v>153</v>
-      </c>
-      <c r="C39" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="B40" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+      <c r="D40" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B41" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C41" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="D41" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2236,142 +2306,142 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
         <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
         <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
       </c>
       <c r="D12" s="1"/>
     </row>
@@ -2380,24 +2450,24 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2418,142 +2488,142 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
         <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
         <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
       </c>
       <c r="D12" s="1"/>
     </row>
@@ -2562,58 +2632,58 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2634,142 +2704,142 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
         <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
         <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
       </c>
       <c r="D12" s="1"/>
     </row>
@@ -2778,18 +2848,18 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2799,7 +2869,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41603806-A543-4947-8607-F0E1E4508892}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -2812,295 +2882,307 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>188</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
         <v>11</v>
-      </c>
-      <c r="C12" t="s">
-        <v>12</v>
       </c>
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" t="s">
-        <v>18</v>
-      </c>
       <c r="D13" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>46</v>
-      </c>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="1"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="B16" t="s">
-        <v>171</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="D16" t="s">
-        <v>172</v>
-      </c>
-      <c r="E16" t="s">
-        <v>176</v>
-      </c>
-      <c r="F16" t="s">
-        <v>101</v>
+      <c r="A16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>191</v>
+      <c r="A17" t="s">
+        <v>180</v>
       </c>
       <c r="B17" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="D17" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E17" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="F17" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
-        <v>194</v>
+      <c r="A18" t="s">
+        <v>181</v>
       </c>
       <c r="B18" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="C18" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="D18" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E18" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="F18" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
-        <v>192</v>
+      <c r="A19" t="s">
+        <v>184</v>
       </c>
       <c r="B19" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="C19" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" t="s">
+        <v>162</v>
+      </c>
+      <c r="E19" t="s">
+        <v>166</v>
+      </c>
+      <c r="F19" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>182</v>
+      </c>
+      <c r="B20" t="s">
+        <v>187</v>
+      </c>
+      <c r="C20" t="s">
+        <v>137</v>
+      </c>
+      <c r="D20" t="s">
+        <v>162</v>
+      </c>
+      <c r="E20" t="s">
+        <v>166</v>
+      </c>
+      <c r="F20" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>185</v>
+      </c>
+      <c r="B21" t="s">
+        <v>187</v>
+      </c>
+      <c r="C21" t="s">
+        <v>143</v>
+      </c>
+      <c r="D21" t="s">
+        <v>162</v>
+      </c>
+      <c r="E21" t="s">
+        <v>166</v>
+      </c>
+      <c r="F21" t="s">
         <v>144</v>
       </c>
-      <c r="D19" t="s">
-        <v>172</v>
-      </c>
-      <c r="E19" t="s">
-        <v>176</v>
-      </c>
-      <c r="F19" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="B20" t="s">
-        <v>171</v>
-      </c>
-      <c r="C20" t="s">
-        <v>150</v>
-      </c>
-      <c r="D20" t="s">
-        <v>172</v>
-      </c>
-      <c r="E20" t="s">
-        <v>176</v>
-      </c>
-      <c r="F20" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="B21" t="s">
-        <v>171</v>
-      </c>
-      <c r="C21" t="s">
-        <v>157</v>
-      </c>
-      <c r="D21" t="s">
-        <v>172</v>
-      </c>
-      <c r="E21" t="s">
-        <v>176</v>
-      </c>
-      <c r="F21" t="s">
-        <v>161</v>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>183</v>
+      </c>
+      <c r="B22" t="s">
+        <v>187</v>
+      </c>
+      <c r="C22" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" t="s">
+        <v>166</v>
+      </c>
+      <c r="F22" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -3121,198 +3203,198 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
         <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
         <v>11</v>
-      </c>
-      <c r="C12" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
         <v>17</v>
-      </c>
-      <c r="C13" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="B16" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B17" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="B18" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3334,27 +3416,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="fe920753-c448-4b18-b0e8-18b73856b91a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fe920753-c448-4b18-b0e8-18b73856b91a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="127cd07f-9ffd-4ce8-b21a-e01c9ecdfd33" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010024F51093868FB24EBD35CDAFD175069E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="84be37977f167f33bd3126630a183308">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fe920753-c448-4b18-b0e8-18b73856b91a" xmlns:ns3="127cd07f-9ffd-4ce8-b21a-e01c9ecdfd33" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="468d2d265cee29b3ccbe510123b8323a" ns2:_="" ns3:_="">
     <xsd:import namespace="fe920753-c448-4b18-b0e8-18b73856b91a"/>
@@ -3573,32 +3634,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90095A14-373E-46B8-A609-CE77E7041A80}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="fe920753-c448-4b18-b0e8-18b73856b91a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="127cd07f-9ffd-4ce8-b21a-e01c9ecdfd33"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9A6A36E-DDA5-4D61-81B4-BE56B2BC85AF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="fe920753-c448-4b18-b0e8-18b73856b91a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fe920753-c448-4b18-b0e8-18b73856b91a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="127cd07f-9ffd-4ce8-b21a-e01c9ecdfd33" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71A7481B-B3C3-451C-BC28-8D07A1B6586A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3615,4 +3672,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9A6A36E-DDA5-4D61-81B4-BE56B2BC85AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90095A14-373E-46B8-A609-CE77E7041A80}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="fe920753-c448-4b18-b0e8-18b73856b91a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="127cd07f-9ffd-4ce8-b21a-e01c9ecdfd33"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Correction of errors in CV and common ontologies data
</commit_message>
<xml_diff>
--- a/SR-dev/metadata/cv-skos-play.xlsx
+++ b/SR-dev/metadata/cv-skos-play.xlsx
@@ -1,24 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aschiltz003\Documents\GitHub\EU-wide-Registry-of-Semantic-Models\SR-dev\metadata\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54F6314B-7565-4FA0-9F8C-C1C2DDF6DFA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Asset" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Agent" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Class" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="ContactPoint" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Document" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Location" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="AssetDistribution" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Concept" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Asset" sheetId="1" r:id="rId1"/>
+    <sheet name="Agent" sheetId="2" r:id="rId2"/>
+    <sheet name="Class" sheetId="3" r:id="rId3"/>
+    <sheet name="ContactPoint" sheetId="4" r:id="rId4"/>
+    <sheet name="Document" sheetId="5" r:id="rId5"/>
+    <sheet name="Location" sheetId="6" r:id="rId6"/>
+    <sheet name="AssetDistribution" sheetId="7" r:id="rId7"/>
+    <sheet name="Concept" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -26,628 +42,605 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>tc={69670AD0-6484-4FFE-A455-3E1E94647EC3}</author>
-  </authors>
-  <commentList>
-    <comment ref="K15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    To be added</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="195">
-  <si>
-    <t xml:space="preserve">ConceptScheme URI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/adms#Asset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PREFIX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/adms#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://publications.europa.eu/resource/authority/corporate-body/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://data.europa.eu/m8g/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dcat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/dcat#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://purl.org/dc/terms/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">foaf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://xmlns.com/foaf/0.1/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">owl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/2002/07/owl#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/dx/prof/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/1999/02/22-rdf-syntax-ns#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vann</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://purl.org/vocab/vann/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xsd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/2001/XMLSchema#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">URI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:contactPoint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:contributor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:creator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:created^^xsd:dateTime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:issued</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:modified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:description@en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:hasImplementation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dcat:distribution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">foaf:homepage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:identifier^^xsd:string</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:isReusedBy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dcat:keyword</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:language</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:lovRank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vann:preferredNamespaceUri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:publisher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:requires</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adms:status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dcat:theme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:title@en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">owl:versionInfo^^xsd:string</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rdf:type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cb:DIGIT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Core Person Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a Person.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.1/voc/core-person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.1/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://publications.europa.eu/resource/authority/language/ENG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core Person Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adms:Asset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Location-Vocabulary/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Core Location Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a location, represented as an address, a geographic name, or a geometry.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Location-Vocabulary/releases/2.1.0/voc/core-location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Location-Vocabulary/releases/2.1.0/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core Location Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Business-Vocabulary/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Core Business Vocabulary is a simplified, reusable and extensible data model that provides a minimum set of classes and properties for legal entities, that is, trading bodies that are formally registered with the relevant authority and that appear in business registers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Business-Vocabulary/releases/2.2.0/voc/core-business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Business-Vocabulary/releases/2.2.0/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core Business Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CCCEV/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Core Criterion an Core Evidence Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of criterion and Evidence.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CCCEV/releases/2.1.0/voc/cccev</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CCCEV/releases/2.1.0/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCCEV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core Criterion and Core Evidence Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CPOV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Core Public Organisation Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a public organisation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CPOV/releases/2.1.1/voc/core-public-organisation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CPOV/releases/2.1.1/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPOV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core Public Organisation Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Core Public Event Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a public event.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Public-Event-Vocabulary/releases/1.1.0/voc/core-public-event</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Public-Event-Vocabulary/releases/1.1.0/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPEV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core Public Event Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.1.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Class URI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://xmlns.com/foaf/0.1/Agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:spatial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIGIT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://publications.europa.eu/resource/authority/country/EUR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">foaf:Agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/2000/01/rdf-schema#Class</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://inspire.ec.europa.eu/ont/ad#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">legal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/legal#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">locn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/locn#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/person#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rdfs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/2000/01/rdf-schema#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rdfs:label@en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rdfs:isDefinedBy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">locn:Address</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rdfs:Class</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Location-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV, https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:ContactPoint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact Point</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV, https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adms:Identifier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identifier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:Location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Location-Vocabulary/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">person:Person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:AdminUnit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Administrative Unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">locn:Geometry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geometry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ad:LocatorDesignator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Locator Designator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:AccountingDocument</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accounting Document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">legal:LegalEntity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legal Entity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:Constraint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constraint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:Criterion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criterion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:Evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:EvidenceType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:EvidenceTypeList</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence Type List</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:InformationConcept</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information Concept</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:InformationRequirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information Requirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:ReferenceFramework</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference Framework</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:Requirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:PublicOrganisation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public Organisation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:Participation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Participation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:PublicEvent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public Event</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://data.europa.eu/m8g/ContactPoint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cv:hasMail^^xsd:string</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIGIT-SEMIC-TEAM@ec.europa.eu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://xmlns.com/foaf/0.1/Document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">foaf:Document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://purl.org/dc/terms/Location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/ns/adms#AssetDistribution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">skos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/2004/02/skos/core#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dcat:downloadURL^^xsd:anyURI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dct:format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prof:hasRole</t>
-  </si>
-  <si>
-    <t xml:space="preserve">amds:AssetDistribution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.1/voc/core-person-ap.ttl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://publications.europa.eu/resource/authority/file-type/RDF_TURTLE</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="196">
+  <si>
+    <t>ConceptScheme URI</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/adms#Asset</t>
+  </si>
+  <si>
+    <t>PREFIX</t>
+  </si>
+  <si>
+    <t>adms</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/adms#</t>
+  </si>
+  <si>
+    <t>cb</t>
+  </si>
+  <si>
+    <t>http://publications.europa.eu/resource/authority/corporate-body/</t>
+  </si>
+  <si>
+    <t>cv</t>
+  </si>
+  <si>
+    <t>http://data.europa.eu/m8g/</t>
+  </si>
+  <si>
+    <t>dcat</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/dcat#</t>
+  </si>
+  <si>
+    <t>dct</t>
+  </si>
+  <si>
+    <t>http://purl.org/dc/terms/</t>
+  </si>
+  <si>
+    <t>foaf</t>
+  </si>
+  <si>
+    <t>http://xmlns.com/foaf/0.1/</t>
+  </si>
+  <si>
+    <t>owl</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/2002/07/owl#</t>
+  </si>
+  <si>
+    <t>prof</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/dx/prof/</t>
+  </si>
+  <si>
+    <t>rdf</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/1999/02/22-rdf-syntax-ns#</t>
+  </si>
+  <si>
+    <t>vann</t>
+  </si>
+  <si>
+    <t>http://purl.org/vocab/vann/</t>
+  </si>
+  <si>
+    <t>xsd</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/2001/XMLSchema#</t>
+  </si>
+  <si>
+    <t>URI</t>
+  </si>
+  <si>
+    <t>cv:contactPoint</t>
+  </si>
+  <si>
+    <t>dct:contributor</t>
+  </si>
+  <si>
+    <t>dct:creator</t>
+  </si>
+  <si>
+    <t>dct:created^^xsd:dateTime</t>
+  </si>
+  <si>
+    <t>dct:issued</t>
+  </si>
+  <si>
+    <t>dct:modified</t>
+  </si>
+  <si>
+    <t>dct:description@en</t>
+  </si>
+  <si>
+    <t>cv:hasImplementation</t>
+  </si>
+  <si>
+    <t>dcat:distribution</t>
+  </si>
+  <si>
+    <t>foaf:homepage</t>
+  </si>
+  <si>
+    <t>dct:identifier^^xsd:string</t>
+  </si>
+  <si>
+    <t>cv:isReusedBy</t>
+  </si>
+  <si>
+    <t>dcat:keyword</t>
+  </si>
+  <si>
+    <t>dct:language</t>
+  </si>
+  <si>
+    <t>cv:lovRank</t>
+  </si>
+  <si>
+    <t>vann:preferredNamespaceUri</t>
+  </si>
+  <si>
+    <t>dct:publisher</t>
+  </si>
+  <si>
+    <t>dct:requires</t>
+  </si>
+  <si>
+    <t>adms:status</t>
+  </si>
+  <si>
+    <t>dcat:theme</t>
+  </si>
+  <si>
+    <t>dct:title@en</t>
+  </si>
+  <si>
+    <t>owl:versionInfo^^xsd:string</t>
+  </si>
+  <si>
+    <t>rdf:type</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/</t>
+  </si>
+  <si>
+    <t>cb:DIGIT</t>
+  </si>
+  <si>
+    <t>The Core Person Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a Person.</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.1/voc/core-person</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.1/</t>
+  </si>
+  <si>
+    <t>CPV</t>
+  </si>
+  <si>
+    <t>http://publications.europa.eu/resource/authority/language/ENG</t>
+  </si>
+  <si>
+    <t>Core Person Vocabulary</t>
+  </si>
+  <si>
+    <t>2.1.1</t>
+  </si>
+  <si>
+    <t>adms:Asset</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Location-Vocabulary/</t>
+  </si>
+  <si>
+    <t>The Core Location Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a location, represented as an address, a geographic name, or a geometry.</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Location-Vocabulary/releases/2.1.0/voc/core-location</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Location-Vocabulary/releases/2.1.0/</t>
+  </si>
+  <si>
+    <t>CLV</t>
+  </si>
+  <si>
+    <t>Core Location Vocabulary</t>
+  </si>
+  <si>
+    <t>2.1.0</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Business-Vocabulary/</t>
+  </si>
+  <si>
+    <t>The Core Business Vocabulary is a simplified, reusable and extensible data model that provides a minimum set of classes and properties for legal entities, that is, trading bodies that are formally registered with the relevant authority and that appear in business registers.</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Business-Vocabulary/releases/2.2.0/voc/core-business</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Business-Vocabulary/releases/2.2.0/</t>
+  </si>
+  <si>
+    <t>CBV</t>
+  </si>
+  <si>
+    <t>Core Business Vocabulary</t>
+  </si>
+  <si>
+    <t>2.2.0</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CCCEV/</t>
+  </si>
+  <si>
+    <t>The Core Criterion an Core Evidence Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of criterion and Evidence.</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CCCEV/releases/2.1.0/voc/cccev</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CCCEV/releases/2.1.0/</t>
+  </si>
+  <si>
+    <t>CCCEV</t>
+  </si>
+  <si>
+    <t>Core Criterion and Core Evidence Vocabulary</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CPOV</t>
+  </si>
+  <si>
+    <t>The Core Public Organisation Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a public organisation.</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CPOV/releases/2.1.1/voc/core-public-organisation</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CPOV/releases/2.1.1/</t>
+  </si>
+  <si>
+    <t>CPOV</t>
+  </si>
+  <si>
+    <t>Core Public Organisation Vocabulary</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
+  </si>
+  <si>
+    <t>The Core Public Event Vocabulary is a simplified, reusable and extensible data model that captures the fundamental characteristics of a public event.</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Public-Event-Vocabulary/releases/1.1.0/voc/core-public-event</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Public-Event-Vocabulary/releases/1.1.0/</t>
+  </si>
+  <si>
+    <t>CPEV</t>
+  </si>
+  <si>
+    <t>Core Public Event Vocabulary</t>
+  </si>
+  <si>
+    <t>1.1.0</t>
+  </si>
+  <si>
+    <t>Class URI</t>
+  </si>
+  <si>
+    <t>http://xmlns.com/foaf/0.1/Agent</t>
+  </si>
+  <si>
+    <t>dct:spatial</t>
+  </si>
+  <si>
+    <t>dct:type</t>
+  </si>
+  <si>
+    <t>DIGIT</t>
+  </si>
+  <si>
+    <t>http://publications.europa.eu/resource/authority/country/EUR</t>
+  </si>
+  <si>
+    <t>foaf:Agent</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/2000/01/rdf-schema#Class</t>
+  </si>
+  <si>
+    <t>ad</t>
+  </si>
+  <si>
+    <t>http://inspire.ec.europa.eu/ont/ad#</t>
+  </si>
+  <si>
+    <t>legal</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/legal#</t>
+  </si>
+  <si>
+    <t>locn</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/locn#</t>
+  </si>
+  <si>
+    <t>person</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/person#</t>
+  </si>
+  <si>
+    <t>rdfs</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/2000/01/rdf-schema#</t>
+  </si>
+  <si>
+    <t>rdfs:label@en</t>
+  </si>
+  <si>
+    <t>rdfs:isDefinedBy</t>
+  </si>
+  <si>
+    <t>locn:Address</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>rdfs:Class</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Location-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV, https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
+  </si>
+  <si>
+    <t>cv:ContactPoint</t>
+  </si>
+  <si>
+    <t>Contact Point</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV, https://semiceu.github.io/Core-Public-Event-Vocabulary/</t>
+  </si>
+  <si>
+    <t>adms:Identifier</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Business-Vocabulary/, https://semiceu.github.io/CPOV</t>
+  </si>
+  <si>
+    <t>dct:Location</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/, https://semiceu.github.io/Core-Location-Vocabulary/</t>
+  </si>
+  <si>
+    <t>person:Person</t>
+  </si>
+  <si>
+    <t>Person</t>
+  </si>
+  <si>
+    <t>cv:AdminUnit</t>
+  </si>
+  <si>
+    <t>Administrative Unit</t>
+  </si>
+  <si>
+    <t>locn:Geometry</t>
+  </si>
+  <si>
+    <t>Geometry</t>
+  </si>
+  <si>
+    <t>ad:LocatorDesignator</t>
+  </si>
+  <si>
+    <t>Locator Designator</t>
+  </si>
+  <si>
+    <t>cv:AccountingDocument</t>
+  </si>
+  <si>
+    <t>Accounting Document</t>
+  </si>
+  <si>
+    <t>legal:LegalEntity</t>
+  </si>
+  <si>
+    <t>Legal Entity</t>
+  </si>
+  <si>
+    <t>cv:Constraint</t>
+  </si>
+  <si>
+    <t>Constraint</t>
+  </si>
+  <si>
+    <t>cv:Criterion</t>
+  </si>
+  <si>
+    <t>Criterion</t>
+  </si>
+  <si>
+    <t>cv:Evidence</t>
+  </si>
+  <si>
+    <t>Evidence</t>
+  </si>
+  <si>
+    <t>cv:EvidenceType</t>
+  </si>
+  <si>
+    <t>Evidence Type</t>
+  </si>
+  <si>
+    <t>cv:EvidenceTypeList</t>
+  </si>
+  <si>
+    <t>Evidence Type List</t>
+  </si>
+  <si>
+    <t>cv:InformationConcept</t>
+  </si>
+  <si>
+    <t>Information Concept</t>
+  </si>
+  <si>
+    <t>cv:InformationRequirement</t>
+  </si>
+  <si>
+    <t>Information Requirement</t>
+  </si>
+  <si>
+    <t>cv:ReferenceFramework</t>
+  </si>
+  <si>
+    <t>Reference Framework</t>
+  </si>
+  <si>
+    <t>cv:Requirement</t>
+  </si>
+  <si>
+    <t>Requirement</t>
+  </si>
+  <si>
+    <t>cv:PublicOrganisation</t>
+  </si>
+  <si>
+    <t>Public Organisation</t>
+  </si>
+  <si>
+    <t>cv:Participation</t>
+  </si>
+  <si>
+    <t>Participation</t>
+  </si>
+  <si>
+    <t>cv:PublicEvent</t>
+  </si>
+  <si>
+    <t>Public Event</t>
+  </si>
+  <si>
+    <t>http://data.europa.eu/m8g/ContactPoint</t>
+  </si>
+  <si>
+    <t>cv:hasMail^^xsd:string</t>
+  </si>
+  <si>
+    <t>DIGIT-SEMIC-TEAM@ec.europa.eu</t>
+  </si>
+  <si>
+    <t>http://xmlns.com/foaf/0.1/Document</t>
+  </si>
+  <si>
+    <t>foaf:Document</t>
+  </si>
+  <si>
+    <t>http://purl.org/dc/terms/Location</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/adms#AssetDistribution</t>
+  </si>
+  <si>
+    <t>skos</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/2004/02/skos/core#</t>
+  </si>
+  <si>
+    <t>dcat:downloadURL^^xsd:anyURI</t>
+  </si>
+  <si>
+    <t>dct:format</t>
+  </si>
+  <si>
+    <t>prof:hasRole</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.1/voc/core-person-ap.ttl</t>
+  </si>
+  <si>
+    <t>http://publications.europa.eu/resource/authority/file-type/RDF_TURTLE</t>
   </si>
   <si>
     <t xml:space="preserve">	http://www.w3.org/ns/dx/prof/role/vocabulary</t>
   </si>
   <si>
-    <t xml:space="preserve">RDF Turtle file of Core Person Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Location-Vocabulary/releases/2.1.0/voc/core-location.ttl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RDF Turtle file of Core Location Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Business-Vocabulary/releases/2.2.0/voc/core-business-ap.ttl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RDF Turtle file of Core Business Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CCCEV/releases/2.1.0/voc/cccev.ttl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RDF Turtle file of Core Criterion and Core Evidence Vocabulary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/CPOV/releases/2.1.1/voc/core-public-organisation-ap.ttl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RDF Turtle file of Core Public Organisation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiceu.github.io/Core-Public-Event-Vocabulary/releases/1.1.0/voc/core-public-event.ttl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RDF Turtle file of Core Public Event</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://www.w3.org/2004/02/skos/core#Concept</t>
-  </si>
-  <si>
-    <t xml:space="preserve">skos:inScheme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">skos:topConceptOf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">skos:Concept</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://publications.europa.eu/resource/authority/file-type/</t>
+    <t>RDF Turtle file of Core Person Vocabulary</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Location-Vocabulary/releases/2.1.0/voc/core-location.ttl</t>
+  </si>
+  <si>
+    <t>RDF Turtle file of Core Location Vocabulary</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Business-Vocabulary/releases/2.2.0/voc/core-business-ap.ttl</t>
+  </si>
+  <si>
+    <t>RDF Turtle file of Core Business Vocabulary</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CCCEV/releases/2.1.0/voc/cccev.ttl</t>
+  </si>
+  <si>
+    <t>RDF Turtle file of Core Criterion and Core Evidence Vocabulary</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/CPOV/releases/2.1.1/voc/core-public-organisation-ap.ttl</t>
+  </si>
+  <si>
+    <t>RDF Turtle file of Core Public Organisation</t>
+  </si>
+  <si>
+    <t>https://semiceu.github.io/Core-Public-Event-Vocabulary/releases/1.1.0/voc/core-public-event.ttl</t>
+  </si>
+  <si>
+    <t>RDF Turtle file of Core Public Event</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/2004/02/skos/core#Concept</t>
+  </si>
+  <si>
+    <t>skos:inScheme</t>
+  </si>
+  <si>
+    <t>skos:topConceptOf</t>
+  </si>
+  <si>
+    <t>skos:Concept</t>
+  </si>
+  <si>
+    <t>http://publications.europa.eu/resource/authority/file-type/</t>
   </si>
   <si>
     <t xml:space="preserve">	http://www.w3.org/ns/dx/prof/role/</t>
   </si>
   <si>
-    <t xml:space="preserve">http://publications.europa.eu/resource/authority/language/</t>
+    <t>http://publications.europa.eu/resource/authority/language/</t>
+  </si>
+  <si>
+    <t>adms:AssetDistribution</t>
+  </si>
+  <si>
+    <t>foaf:name@en</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -656,40 +649,20 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u val="single"/>
+      <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
@@ -697,7 +670,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -714,13 +687,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.7999"/>
+        <fgColor theme="6" tint="0.79989013336588644"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -728,81 +701,35 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -861,47 +788,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
     <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -909,12 +852,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -943,7 +886,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -964,7 +907,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1015,7 +958,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1033,49 +976,48 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X21"/>
-  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="10.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="24.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="23.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="58.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="9.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="27.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="11.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="10.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="20.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="14.33"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="24" style="1" width="11.56"/>
+    <col min="1" max="1" width="50.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20.109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23.6640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12.88671875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5546875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="58.5546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="9.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="27.33203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="12" style="1" customWidth="1"/>
+    <col min="19" max="19" width="11" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.109375" style="1" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="20.5546875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="14.33203125" style="1" customWidth="1"/>
+    <col min="24" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1083,7 +1025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1094,7 +1036,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -1105,7 +1047,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1116,7 +1058,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1127,7 +1069,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -1138,7 +1080,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -1149,7 +1091,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -1160,7 +1102,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -1171,7 +1113,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1182,7 +1124,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -1193,7 +1135,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -1204,7 +1146,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>2</v>
       </c>
@@ -1215,7 +1157,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
@@ -1289,7 +1231,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>49</v>
       </c>
@@ -1300,8 +1242,8 @@
       <c r="D16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <f aca="false">DATE(2024,5,6)</f>
+      <c r="E16" s="6">
+        <f t="shared" ref="E16:E21" si="0">DATE(2024,5,6)</f>
         <v>45418</v>
       </c>
       <c r="H16" s="1" t="s">
@@ -1335,7 +1277,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>59</v>
       </c>
@@ -1345,8 +1287,8 @@
       <c r="D17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E17" s="6" t="n">
-        <f aca="false">DATE(2024,5,6)</f>
+      <c r="E17" s="6">
+        <f t="shared" si="0"/>
         <v>45418</v>
       </c>
       <c r="H17" s="1" t="s">
@@ -1380,7 +1322,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>66</v>
       </c>
@@ -1390,8 +1332,8 @@
       <c r="D18" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="6" t="n">
-        <f aca="false">DATE(2024,5,6)</f>
+      <c r="E18" s="6">
+        <f t="shared" si="0"/>
         <v>45418</v>
       </c>
       <c r="H18" s="1" t="s">
@@ -1425,7 +1367,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>73</v>
       </c>
@@ -1435,8 +1377,8 @@
       <c r="D19" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="6" t="n">
-        <f aca="false">DATE(2024,5,6)</f>
+      <c r="E19" s="6">
+        <f t="shared" si="0"/>
         <v>45418</v>
       </c>
       <c r="H19" s="1" t="s">
@@ -1470,7 +1412,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>79</v>
       </c>
@@ -1480,8 +1422,8 @@
       <c r="D20" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E20" s="6" t="n">
-        <f aca="false">DATE(2024,5,6)</f>
+      <c r="E20" s="6">
+        <f t="shared" si="0"/>
         <v>45418</v>
       </c>
       <c r="H20" s="1" t="s">
@@ -1515,7 +1457,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>85</v>
       </c>
@@ -1525,8 +1467,8 @@
       <c r="D21" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E21" s="6" t="n">
-        <f aca="false">DATE(2024,5,6)</f>
+      <c r="E21" s="6">
+        <f t="shared" si="0"/>
         <v>45418</v>
       </c>
       <c r="H21" s="1" t="s">
@@ -1561,34 +1503,25 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="61.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.67"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="8.54"/>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
@@ -1597,7 +1530,7 @@
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1609,7 +1542,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -1621,7 +1554,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1633,7 +1566,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1645,7 +1578,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -1657,7 +1590,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -1669,7 +1602,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -1681,7 +1614,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -1693,7 +1626,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1705,7 +1638,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -1717,7 +1650,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -1729,15 +1662,15 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>46</v>
+        <v>195</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>94</v>
@@ -1749,7 +1682,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
@@ -1764,34 +1697,26 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="8.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="8.88"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="1" width="8.54"/>
+    <col min="1" max="1" width="31.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="40.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" style="1" customWidth="1"/>
+    <col min="5" max="6" width="8.5546875" style="1"/>
+    <col min="7" max="8" width="8.88671875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
@@ -1800,7 +1725,7 @@
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1812,7 +1737,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -1824,7 +1749,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1836,7 +1761,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1848,7 +1773,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -1860,7 +1785,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -1872,7 +1797,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -1884,7 +1809,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -1896,7 +1821,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1908,7 +1833,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -1920,7 +1845,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -1932,7 +1857,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>2</v>
       </c>
@@ -1944,7 +1869,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>2</v>
       </c>
@@ -1956,7 +1881,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>2</v>
       </c>
@@ -1968,7 +1893,7 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>2</v>
       </c>
@@ -1980,7 +1905,7 @@
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>2</v>
       </c>
@@ -1992,7 +1917,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>25</v>
       </c>
@@ -2006,7 +1931,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>112</v>
       </c>
@@ -2020,7 +1945,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>116</v>
       </c>
@@ -2034,7 +1959,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>119</v>
       </c>
@@ -2048,7 +1973,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>122</v>
       </c>
@@ -2062,7 +1987,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>125</v>
       </c>
@@ -2076,7 +2001,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>127</v>
       </c>
@@ -2090,7 +2015,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>129</v>
       </c>
@@ -2104,7 +2029,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>131</v>
       </c>
@@ -2118,7 +2043,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>133</v>
       </c>
@@ -2132,7 +2057,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>135</v>
       </c>
@@ -2146,7 +2071,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>137</v>
       </c>
@@ -2160,7 +2085,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>139</v>
       </c>
@@ -2174,7 +2099,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>141</v>
       </c>
@@ -2188,7 +2113,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>143</v>
       </c>
@@ -2202,7 +2127,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>145</v>
       </c>
@@ -2216,7 +2141,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>147</v>
       </c>
@@ -2230,7 +2155,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>149</v>
       </c>
@@ -2244,7 +2169,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>151</v>
       </c>
@@ -2258,7 +2183,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>153</v>
       </c>
@@ -2272,7 +2197,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>155</v>
       </c>
@@ -2286,7 +2211,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>157</v>
       </c>
@@ -2300,7 +2225,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>159</v>
       </c>
@@ -2315,32 +2240,24 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="8.54"/>
+    <col min="1" max="1" width="43.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="38.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
@@ -2349,7 +2266,7 @@
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2361,7 +2278,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2373,7 +2290,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2385,7 +2302,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -2397,7 +2314,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -2409,7 +2326,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -2421,7 +2338,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -2433,7 +2350,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -2445,7 +2362,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -2457,7 +2374,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -2469,7 +2386,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -2481,10 +2398,10 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
@@ -2495,7 +2412,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
@@ -2507,32 +2424,24 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="67.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="8.54"/>
+    <col min="1" max="1" width="67.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="35.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
@@ -2541,7 +2450,7 @@
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2553,7 +2462,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2565,7 +2474,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2577,7 +2486,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -2589,7 +2498,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -2601,7 +2510,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -2613,7 +2522,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -2625,7 +2534,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -2637,7 +2546,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -2649,7 +2558,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -2661,7 +2570,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -2673,10 +2582,10 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
@@ -2684,7 +2593,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
@@ -2692,7 +2601,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>62</v>
       </c>
@@ -2700,7 +2609,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>69</v>
       </c>
@@ -2708,7 +2617,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>76</v>
       </c>
@@ -2716,7 +2625,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>82</v>
       </c>
@@ -2724,7 +2633,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>88</v>
       </c>
@@ -2733,32 +2642,24 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="62.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="8.54"/>
+    <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="62.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
@@ -2767,7 +2668,7 @@
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2779,7 +2680,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2791,7 +2692,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2803,7 +2704,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -2815,7 +2716,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -2827,7 +2728,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -2839,7 +2740,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -2851,7 +2752,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -2863,7 +2764,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -2875,7 +2776,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -2887,7 +2788,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -2899,10 +2800,10 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
@@ -2910,7 +2811,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>97</v>
       </c>
@@ -2919,34 +2820,26 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="67.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.56"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="8.54"/>
+    <col min="1" max="1" width="18.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="67.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="25.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.5546875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
@@ -2955,7 +2848,7 @@
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2967,7 +2860,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2979,7 +2872,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2991,7 +2884,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -3003,7 +2896,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -3015,7 +2908,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -3027,7 +2920,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -3039,7 +2932,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -3051,7 +2944,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -3063,7 +2956,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -3075,7 +2968,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -3087,7 +2980,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>2</v>
       </c>
@@ -3099,7 +2992,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>2</v>
       </c>
@@ -3111,7 +3004,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
@@ -3131,161 +3024,153 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>187</v>
-      </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="62.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="38.56"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="8.54"/>
+    <col min="1" max="1" width="42.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="48.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="62.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="38.5546875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -3296,7 +3181,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -3307,7 +3192,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3318,7 +3203,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
@@ -3329,7 +3214,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
@@ -3340,7 +3225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -3351,7 +3236,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -3362,7 +3247,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -3373,7 +3258,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -3384,7 +3269,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>2</v>
       </c>
@@ -3395,7 +3280,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
@@ -3406,7 +3291,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>2</v>
       </c>
@@ -3417,7 +3302,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
@@ -3425,75 +3310,70 @@
         <v>48</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="D15" s="4" t="s">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="C16" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="B17" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>55</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1" r:id="rId1" location="Concept" display="http://www.w3.org/2004/02/skos/core#Concept"/>
-    <hyperlink ref="C3" r:id="rId2" display="http://publications.europa.eu/resource/authority/corporate-body/"/>
-    <hyperlink ref="A16" r:id="rId3" display="http://publications.europa.eu/resource/authority/file-type/RDF_TURTLE"/>
-    <hyperlink ref="C16" r:id="rId4" display="http://publications.europa.eu/resource/authority/file-type/"/>
-    <hyperlink ref="D16" r:id="rId5" display="http://publications.europa.eu/resource/authority/file-type/"/>
-    <hyperlink ref="A17" r:id="rId6" location="Role:vocabulary" display="&#9;http://www.w3.org/ns/dx/prof/role/vocabulary"/>
-    <hyperlink ref="C17" r:id="rId7" location="Role:vocabulary" display="&#9;http://www.w3.org/ns/dx/prof/role/"/>
-    <hyperlink ref="D17" r:id="rId8" location="Role:vocabulary" display="&#9;http://www.w3.org/ns/dx/prof/role/"/>
-    <hyperlink ref="A18" r:id="rId9" display="http://publications.europa.eu/resource/authority/language/ENG"/>
-    <hyperlink ref="C18" r:id="rId10" display="http://publications.europa.eu/resource/authority/language/"/>
-    <hyperlink ref="D18" r:id="rId11" display="http://publications.europa.eu/resource/authority/language/"/>
+    <hyperlink ref="B1" r:id="rId1" location="Concept" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
+    <hyperlink ref="A16" r:id="rId3" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
+    <hyperlink ref="C16" r:id="rId4" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
+    <hyperlink ref="D16" r:id="rId5" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
+    <hyperlink ref="A17" r:id="rId6" location="Role:vocabulary" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
+    <hyperlink ref="C17" r:id="rId7" location="Role:vocabulary" xr:uid="{00000000-0004-0000-0700-000006000000}"/>
+    <hyperlink ref="D17" r:id="rId8" location="Role:vocabulary" xr:uid="{00000000-0004-0000-0700-000007000000}"/>
+    <hyperlink ref="A18" r:id="rId9" xr:uid="{00000000-0004-0000-0700-000008000000}"/>
+    <hyperlink ref="C18" r:id="rId10" xr:uid="{00000000-0004-0000-0700-000009000000}"/>
+    <hyperlink ref="D18" r:id="rId11" xr:uid="{00000000-0004-0000-0700-00000A000000}"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -3716,27 +3596,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="fe920753-c448-4b18-b0e8-18b73856b91a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fe920753-c448-4b18-b0e8-18b73856b91a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="127cd07f-9ffd-4ce8-b21a-e01c9ecdfd33" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71A7481B-B3C3-451C-BC28-8D07A1B6586A}">
   <ds:schemaRefs>
@@ -3754,29 +3613,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9A6A36E-DDA5-4D61-81B4-BE56B2BC85AF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90095A14-373E-46B8-A609-CE77E7041A80}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="fe920753-c448-4b18-b0e8-18b73856b91a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="127cd07f-9ffd-4ce8-b21a-e01c9ecdfd33"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>